<commit_message>
did lots of correcting
</commit_message>
<xml_diff>
--- a/2_ADAS_ECU/4.1_ADAS_ECU_revA (ORIN NX)/0_CALCS/POWER_BUDGET.xlsx
+++ b/2_ADAS_ECU/4.1_ADAS_ECU_revA (ORIN NX)/0_CALCS/POWER_BUDGET.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\se097192\Documents\0_BRZ\1_BRZ_HARDWARE\2_ADAS_ECU\4.1_ADAS_ECU_revA (ORIN NX)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BRZ\1_BRZ_HARDWARE\2_ADAS_ECU\4.1_ADAS_ECU_revA (ORIN NX)\0_CALCS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21647E18-5CC5-4872-B278-9D4093B37320}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DF9814-8213-4EF4-A16D-49ABFEEC7329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F9C4DBE3-62FA-4DEE-9748-8747E0CAF855}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="40">
   <si>
     <t>Device</t>
   </si>
@@ -169,6 +169,12 @@
   </si>
   <si>
     <t>Guess, assuming .5A draw</t>
+  </si>
+  <si>
+    <t>&lt;-- current draw at 12V</t>
+  </si>
+  <si>
+    <t>Rounded up from 5W which is what some 1TB Gen4 SSDs can run at</t>
   </si>
 </sst>
 </file>
@@ -226,10 +232,10 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -825,11 +831,11 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
       <c r="D14">
         <f>SUMPRODUCT($B$3:$B$12,D3:D12)</f>
         <v>9</v>
@@ -864,11 +870,11 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
       <c r="D15">
         <f>D14/2</f>
         <v>4.5</v>
@@ -903,11 +909,11 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
       <c r="D16">
         <f>CEILING(D15, 5)</f>
         <v>5</v>
@@ -941,11 +947,11 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
       <c r="D17">
         <f>CEILING(D16/2,1)</f>
         <v>3</v>
@@ -1002,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75AC54BA-5AF0-4249-A95B-01DDC1DC18C5}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.5703125" bestFit="1" customWidth="1"/>
@@ -1012,21 +1018,22 @@
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="6" max="6" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="3"/>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="2"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="3"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1048,9 +1055,9 @@
       <c r="G2" t="s">
         <v>28</v>
       </c>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1063,12 +1070,12 @@
       <c r="D3">
         <v>40</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1078,15 +1085,18 @@
       <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
       <c r="F4">
-        <v>10</v>
-      </c>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="J4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1096,15 +1106,15 @@
       <c r="C5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
       <c r="F5">
-        <v>10</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1114,15 +1124,15 @@
       <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
       <c r="F6">
         <v>3</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1135,12 +1145,12 @@
       <c r="D7">
         <v>6</v>
       </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -1150,15 +1160,15 @@
       <c r="C8" t="s">
         <v>26</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="2"/>
       <c r="E8">
         <v>15</v>
       </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -1168,15 +1178,15 @@
       <c r="C9" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="2"/>
       <c r="E9">
-        <v>2</v>
-      </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -1186,15 +1196,15 @@
       <c r="C10" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
       <c r="F10">
-        <v>5</v>
-      </c>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1204,15 +1214,15 @@
       <c r="C11" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
       <c r="G11">
         <v>24</v>
       </c>
-      <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -1222,84 +1232,91 @@
       <c r="C12" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
       <c r="G12">
-        <v>10</v>
-      </c>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
       <c r="D14">
         <f t="shared" ref="D14:G14" si="0">SUMPRODUCT($B$3:$B$12,D3:D12)</f>
         <v>88</v>
       </c>
       <c r="E14">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F14">
         <f>SUMPRODUCT($B$3:$B$12,F3:F12)</f>
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H14">
         <f>SUM(D14:G14)</f>
-        <v>180</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
       <c r="D15">
         <f>D14/12</f>
         <v>7.333333333333333</v>
       </c>
       <c r="E15">
         <f>E14/5</f>
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="F15">
         <f>F14/3.3</f>
-        <v>9.3939393939393945</v>
+        <v>6.0606060606060606</v>
       </c>
       <c r="G15">
         <f>G14/12</f>
-        <v>3.6666666666666665</v>
+        <v>3.3333333333333335</v>
       </c>
       <c r="H15">
         <f>SUM(D15:G15)</f>
-        <v>23.793939393939393</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+        <v>19.927272727272726</v>
+      </c>
+      <c r="I15">
+        <f>H14/12</f>
+        <v>13.666666666666666</v>
+      </c>
+      <c r="J15" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
       <c r="D16">
         <f>CEILING(D15, 5)</f>
         <v>10</v>
@@ -1322,11 +1339,11 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
       <c r="D17">
         <f t="shared" ref="D17:G17" si="2">CEILING(D16/2,1)</f>
         <v>5</v>

</xml_diff>